<commit_message>
Fix Chair 06 upholstery, correct dimensions, split Storage 29 variants, refine product card layout
- Chair 06 A1: correct LE->FB upholstery code (costing is fabric, not leather);
  rename images in both projects, update database code, tag now reads "Teak + Fabric"
- Correct dimensions from updated Product Dimensions.xlsx: Sofa 28 A1 (205x75x84,
  SH-42) and Bed 27 B1 (281x215x110), which had been wrongly copied from siblings
- Split Storage 29 into two real variants: Storage 29 C1 (Umang, 129x35x80, 54k)
  and Storage 29 C2 (Modern Times, 149x42x181, 149k) with its own image + row,
  resolving the collision where MT showed Umang's smaller item
- Product cards: "Starting at Rs X" wording (drop the + suffix), two-column body
  layout so title/dimensions stack tight on the left independent of the taller
  price/material block on the right
- Reserve top-right nav padding so the fixed home pill no longer overlaps the
  edition mark on the hero
- Regenerate umang.html and modern-times.html
</commit_message>
<xml_diff>
--- a/Product_Database.xlsx
+++ b/Product_Database.xlsx
@@ -1619,7 +1619,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chair 06 A1 [1S-LE-N]</t>
+          <t>Chair 06 A1 [1S-FB-N]</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>255</v>
+        <v>205</v>
       </c>
       <c r="E52" t="n">
         <v>75</v>
@@ -2764,7 +2764,7 @@
         <v>84</v>
       </c>
       <c r="G52" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
@@ -2830,10 +2830,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="E54" t="n">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F54" t="n">
         <v>110</v>
@@ -2853,10 +2853,33 @@
       </c>
     </row>
     <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Living</t>
+        </is>
+      </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>product is in theme 1 &amp; umang</t>
-        </is>
+          <t>Storage 29 C2 [STD-XX-N]</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Storage 29 C2</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>149</v>
+      </c>
+      <c r="E55" t="n">
+        <v>42</v>
+      </c>
+      <c r="F55" t="n">
+        <v>181</v>
+      </c>
+      <c r="I55">
+        <f>D55 &amp; "cm x " &amp; E55 &amp; "cm x " &amp; F55 &amp; "cm (H) x SH-" &amp; G55 &amp; "cm"</f>
+        <v/>
       </c>
       <c r="K55" s="6" t="inlineStr">
         <is>
@@ -2865,8 +2888,11 @@
       </c>
       <c r="L55" s="6" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R55" t="n">
+        <v>149000</v>
       </c>
     </row>
     <row r="56">

</xml_diff>